<commit_message>
Update model code, visualization scripts, and clean up documentation files
</commit_message>
<xml_diff>
--- a/data/SAM.xlsx
+++ b/data/SAM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://solisservices-my.sharepoint.com/personal/b_jammeh_uu_nl/Documents/Documents/CGE_Model/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimibit-my.sharepoint.com/personal/b_jammeh_campus_unimib_it/Documents/Desktop/MODELLING/Italian_cge_model/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_BB282D52714AD3D7C892F41848578E2F62974E10" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75FD3A83-02E8-4544-824D-ADC5E4C3B447}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_BB282D52714AD3D7C892F41848578E2F62974E10" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30793FD7-DDDE-4E50-827A-ECC6CBE3C4BA}"/>
   <bookViews>
-    <workbookView xWindow="29940" yWindow="1140" windowWidth="38700" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5070" yWindow="5070" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SAM" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,6 @@
     <t>Industry</t>
   </si>
   <si>
-    <t>Electricity</t>
-  </si>
-  <si>
     <t>Gas</t>
   </si>
   <si>
@@ -86,6 +83,9 @@
   </si>
   <si>
     <t>Rest of World</t>
+  </si>
+  <si>
+    <t>Renewables</t>
   </si>
 </sst>
 </file>
@@ -126,10 +126,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -435,84 +434,86 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.81640625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="14.08984375" customWidth="1"/>
-    <col min="14" max="14" width="19.81640625" customWidth="1"/>
-    <col min="15" max="15" width="18.1796875" customWidth="1"/>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="5" max="5" width="7.5703125" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" customWidth="1"/>
+    <col min="14" max="14" width="19.85546875" customWidth="1"/>
+    <col min="15" max="15" width="18.140625" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2">
@@ -582,8 +583,8 @@
         <v>21075.189544238809</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3">
@@ -653,9 +654,9 @@
         <v>278714.71256760613</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -667,7 +668,7 @@
         <v>4791.8187368748086</v>
       </c>
       <c r="E4">
-        <v>417.62934296818872</v>
+        <v>417.62934296818901</v>
       </c>
       <c r="F4">
         <v>14767.412830566591</v>
@@ -724,9 +725,9 @@
         <v>11595.38182831047</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>3</v>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="B5">
         <v>15.002047234564779</v>
@@ -795,9 +796,9 @@
         <v>7109.9300444108303</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B6">
         <v>9.2811656461551646</v>
@@ -866,9 +867,9 @@
         <v>79862.059058341736</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>5</v>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B7">
         <v>12.144060115094209</v>
@@ -937,9 +938,9 @@
         <v>4558.2047872301473</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>6</v>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="B8">
         <v>0.65023014221916942</v>
@@ -1008,9 +1009,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>7</v>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1079,9 +1080,9 @@
         <v>499.99746909545797</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>8</v>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="B10">
         <v>2.5713261687246649</v>
@@ -1150,9 +1151,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -1221,9 +1222,9 @@
         <v>721.48484351179059</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>10</v>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="B12">
         <v>27972.282555442001</v>
@@ -1292,9 +1293,9 @@
         <v>64848.749056693603</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>11</v>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="B13">
         <v>7845.7379975937874</v>
@@ -1363,9 +1364,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>12</v>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="B14">
         <v>7362.2603638104592</v>
@@ -1434,9 +1435,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>13</v>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1505,9 +1506,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>14</v>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -1576,9 +1577,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>15</v>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1647,9 +1648,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>16</v>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>15</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1718,9 +1719,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>17</v>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1789,9 +1790,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>18</v>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1860,9 +1861,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>19</v>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1931,9 +1932,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
-        <v>20</v>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -2002,9 +2003,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
-        <v>21</v>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="B23">
         <v>3412.0020276557671</v>

</xml_diff>